<commit_message>
Sprint 3.5 - engine de regras parametrizadas, parser, registry e handlers iniciais
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://spsenacbr-my.sharepoint.com/personal/guilherme_odrumond_sp_senac_br/Documents/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{F279B3AB-2542-4CCB-9533-5B948901721C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{992FF7D5-03DD-496D-9297-B5DB3D39A2D1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67659373-BBB2-4118-B6E4-D0D0241B1A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -465,193 +465,193 @@
     <t>CHSA_BLOCO_MINIMO</t>
   </si>
   <si>
+    <t>CNST_COMPLEMENTO_POSICAO</t>
+  </si>
+  <si>
+    <t>BORDA</t>
+  </si>
+  <si>
+    <t>POR_MAX_CONSECUTIVAS</t>
+  </si>
+  <si>
+    <t>MAT_PARES</t>
+  </si>
+  <si>
+    <t>MAT_DIAS_DIFERENTES</t>
+  </si>
+  <si>
+    <t>PROJ_DIA</t>
+  </si>
+  <si>
+    <t>TER</t>
+  </si>
+  <si>
+    <t>PROJ_AULA_INICIAL</t>
+  </si>
+  <si>
+    <t>PROJ_AULA_FINAL</t>
+  </si>
+  <si>
+    <t>Par</t>
+  </si>
+  <si>
+    <t>Especialidade_1</t>
+  </si>
+  <si>
+    <t>Especialidade_2</t>
+  </si>
+  <si>
+    <t>PP_LEST_01</t>
+  </si>
+  <si>
+    <t>PP_CHSA_01</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>BLOCO_OTIMO</t>
+  </si>
+  <si>
+    <t>BLOCO_ACEITAVEL</t>
+  </si>
+  <si>
+    <t>BLOCO_MINIMO</t>
+  </si>
+  <si>
+    <t>COMPLEMENTO</t>
+  </si>
+  <si>
+    <t>POSICAO_COMPLEMENTO</t>
+  </si>
+  <si>
+    <t>MAX_POR_CONSECUTIVAS</t>
+  </si>
+  <si>
+    <t>DUPLAS</t>
+  </si>
+  <si>
+    <t>DIAS_DIFERENTES</t>
+  </si>
+  <si>
+    <t>FIXO</t>
+  </si>
+  <si>
+    <t>TER1-TER4</t>
+  </si>
+  <si>
+    <t>PADRAO_2+2</t>
+  </si>
+  <si>
+    <t>Dia</t>
+  </si>
+  <si>
+    <t>Aula</t>
+  </si>
+  <si>
+    <t>SEG</t>
+  </si>
+  <si>
+    <t>QUA</t>
+  </si>
+  <si>
+    <t>SEX</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>Tecnologia</t>
+  </si>
+  <si>
+    <t>Negocios</t>
+  </si>
+  <si>
+    <t>Multimidia</t>
+  </si>
+  <si>
+    <t>Parâmetro</t>
+  </si>
+  <si>
+    <t>MAX_TIME_SECONDS</t>
+  </si>
+  <si>
+    <t>RANDOM_SEED</t>
+  </si>
+  <si>
+    <t>NUM_WORKERS</t>
+  </si>
+  <si>
+    <t>PESO_CONFLITO_DOCENTE</t>
+  </si>
+  <si>
+    <t>PESO_CONTIGUIDADE</t>
+  </si>
+  <si>
+    <t>PESO_CHSA_BLOCO6</t>
+  </si>
+  <si>
+    <t>PESO_CNST_BLOCO5</t>
+  </si>
+  <si>
+    <t>PESO_LEST_BLOCO6</t>
+  </si>
+  <si>
+    <t>Objetivo</t>
+  </si>
+  <si>
+    <t>Peso</t>
+  </si>
+  <si>
+    <t>CONFLITO_DOCENTE</t>
+  </si>
+  <si>
+    <t>MUDANCA_COMPONENTE</t>
+  </si>
+  <si>
+    <t>BLOCO_CHSA</t>
+  </si>
+  <si>
+    <t>BLOCO_CNST</t>
+  </si>
+  <si>
+    <t>BLOCO_LEST</t>
+  </si>
+  <si>
+    <t>MAX_DIAS_PROF</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Nível</t>
+  </si>
+  <si>
+    <t>Área A</t>
+  </si>
+  <si>
+    <t>Área B</t>
+  </si>
+  <si>
+    <t>Custo</t>
+  </si>
+  <si>
+    <t>TEC</t>
+  </si>
+  <si>
+    <t>NEG</t>
+  </si>
+  <si>
+    <t>COESAO_AREAS</t>
+  </si>
+  <si>
+    <t>FRAGMENTACAO_PROF</t>
+  </si>
+  <si>
     <t>CNST_COMPLEMENTO</t>
-  </si>
-  <si>
-    <t>CNST_COMPLEMENTO_POSICAO</t>
-  </si>
-  <si>
-    <t>BORDA</t>
-  </si>
-  <si>
-    <t>POR_MAX_CONSECUTIVAS</t>
-  </si>
-  <si>
-    <t>MAT_PARES</t>
-  </si>
-  <si>
-    <t>MAT_DIAS_DIFERENTES</t>
-  </si>
-  <si>
-    <t>PROJ_DIA</t>
-  </si>
-  <si>
-    <t>TER</t>
-  </si>
-  <si>
-    <t>PROJ_AULA_INICIAL</t>
-  </si>
-  <si>
-    <t>PROJ_AULA_FINAL</t>
-  </si>
-  <si>
-    <t>Par</t>
-  </si>
-  <si>
-    <t>Especialidade_1</t>
-  </si>
-  <si>
-    <t>Especialidade_2</t>
-  </si>
-  <si>
-    <t>PP_LEST_01</t>
-  </si>
-  <si>
-    <t>PP_CHSA_01</t>
-  </si>
-  <si>
-    <t>Tipo</t>
-  </si>
-  <si>
-    <t>BLOCO_OTIMO</t>
-  </si>
-  <si>
-    <t>BLOCO_ACEITAVEL</t>
-  </si>
-  <si>
-    <t>BLOCO_MINIMO</t>
-  </si>
-  <si>
-    <t>COMPLEMENTO</t>
-  </si>
-  <si>
-    <t>POSICAO_COMPLEMENTO</t>
-  </si>
-  <si>
-    <t>MAX_POR_CONSECUTIVAS</t>
-  </si>
-  <si>
-    <t>DUPLAS</t>
-  </si>
-  <si>
-    <t>DIAS_DIFERENTES</t>
-  </si>
-  <si>
-    <t>FIXO</t>
-  </si>
-  <si>
-    <t>TER1-TER4</t>
-  </si>
-  <si>
-    <t>PADRAO_2+2</t>
-  </si>
-  <si>
-    <t>Dia</t>
-  </si>
-  <si>
-    <t>Aula</t>
-  </si>
-  <si>
-    <t>SEG</t>
-  </si>
-  <si>
-    <t>QUA</t>
-  </si>
-  <si>
-    <t>SEX</t>
-  </si>
-  <si>
-    <t>Area</t>
-  </si>
-  <si>
-    <t>Tecnologia</t>
-  </si>
-  <si>
-    <t>Negocios</t>
-  </si>
-  <si>
-    <t>Multimidia</t>
-  </si>
-  <si>
-    <t>Parâmetro</t>
-  </si>
-  <si>
-    <t>MAX_TIME_SECONDS</t>
-  </si>
-  <si>
-    <t>RANDOM_SEED</t>
-  </si>
-  <si>
-    <t>NUM_WORKERS</t>
-  </si>
-  <si>
-    <t>PESO_CONFLITO_DOCENTE</t>
-  </si>
-  <si>
-    <t>PESO_CONTIGUIDADE</t>
-  </si>
-  <si>
-    <t>PESO_CHSA_BLOCO6</t>
-  </si>
-  <si>
-    <t>PESO_CNST_BLOCO5</t>
-  </si>
-  <si>
-    <t>PESO_LEST_BLOCO6</t>
-  </si>
-  <si>
-    <t>Objetivo</t>
-  </si>
-  <si>
-    <t>Peso</t>
-  </si>
-  <si>
-    <t>CONFLITO_DOCENTE</t>
-  </si>
-  <si>
-    <t>MUDANCA_COMPONENTE</t>
-  </si>
-  <si>
-    <t>BLOCO_CHSA</t>
-  </si>
-  <si>
-    <t>BLOCO_CNST</t>
-  </si>
-  <si>
-    <t>BLOCO_LEST</t>
-  </si>
-  <si>
-    <t>MAX_DIAS_PROF</t>
-  </si>
-  <si>
-    <t>Ativo</t>
-  </si>
-  <si>
-    <t>s</t>
-  </si>
-  <si>
-    <t>Nível</t>
-  </si>
-  <si>
-    <t>Área A</t>
-  </si>
-  <si>
-    <t>Área B</t>
-  </si>
-  <si>
-    <t>Custo</t>
-  </si>
-  <si>
-    <t>TEC</t>
-  </si>
-  <si>
-    <t>NEG</t>
-  </si>
-  <si>
-    <t>COESAO_AREAS</t>
-  </si>
-  <si>
-    <t>FRAGMENTACAO_PROF</t>
   </si>
 </sst>
 </file>
@@ -894,7 +894,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>138</v>
@@ -902,7 +902,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B2" s="1">
         <v>1800</v>
@@ -910,7 +910,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B3" s="1">
         <v>42</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B4" s="1">
         <v>16</v>
@@ -926,7 +926,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B5" s="1">
         <v>500</v>
@@ -934,7 +934,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B6" s="1">
         <v>40</v>
@@ -942,7 +942,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B7" s="1">
         <v>100</v>
@@ -950,7 +950,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B8" s="1">
         <v>80</v>
@@ -958,7 +958,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B9" s="1">
         <v>60</v>
@@ -984,7 +984,7 @@
         <v>38</v>
       </c>
       <c r="B1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>138</v>
@@ -995,7 +995,7 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C2" s="1">
         <v>6</v>
@@ -1006,7 +1006,7 @@
         <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C3" s="1">
         <v>5</v>
@@ -1017,7 +1017,7 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
@@ -1028,7 +1028,7 @@
         <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>96</v>
@@ -1039,10 +1039,10 @@
         <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1050,7 +1050,7 @@
         <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
@@ -1061,7 +1061,7 @@
         <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C8" s="1">
         <v>2</v>
@@ -1072,7 +1072,7 @@
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
@@ -1083,10 +1083,10 @@
         <v>127</v>
       </c>
       <c r="B10" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1105,7 +1105,7 @@
         <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>7</v>
@@ -1127,15 +1127,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1143,7 +1143,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1159,7 +1159,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
@@ -1167,7 +1167,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B6" s="1">
         <v>5</v>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B7" s="1">
         <v>6</v>
@@ -1183,7 +1183,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B8" s="1">
         <v>1</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B10" s="1">
         <v>3</v>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B11" s="1">
         <v>4</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B13" s="1">
         <v>6</v>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B14" s="1">
         <v>1</v>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B15" s="1">
         <v>2</v>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B16" s="1">
         <v>3</v>
@@ -1255,7 +1255,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B17" s="1">
         <v>4</v>
@@ -1263,7 +1263,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B18" s="1">
         <v>5</v>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -1327,7 +1327,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B26" s="1">
         <v>1</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B27" s="1">
         <v>2</v>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B28" s="1">
         <v>3</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B29" s="1">
         <v>4</v>
@@ -1359,7 +1359,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B30" s="1">
         <v>5</v>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B31" s="1">
         <v>6</v>
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1401,7 +1401,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1409,7 +1409,7 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1417,7 +1417,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1425,7 +1425,7 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1433,7 +1433,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1441,7 +1441,7 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1457,21 +1457,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" t="s">
         <v>198</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>199</v>
-      </c>
-      <c r="C1" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1479,10 +1479,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -1512,10 +1512,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B6" t="s">
         <v>201</v>
-      </c>
-      <c r="B6" t="s">
-        <v>202</v>
       </c>
       <c r="C6">
         <v>80</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
@@ -1918,7 +1918,7 @@
         <v>40</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1938,7 +1938,7 @@
         <v>4</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1958,7 +1958,7 @@
         <v>4</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1978,7 +1978,7 @@
         <v>4</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1998,7 +1998,7 @@
         <v>4</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2018,7 +2018,7 @@
         <v>4</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2038,7 +2038,7 @@
         <v>4</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,7 +2058,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2078,7 +2078,7 @@
         <v>4</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2098,7 +2098,7 @@
         <v>3</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2118,7 +2118,7 @@
         <v>4</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2138,7 +2138,7 @@
         <v>3</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2158,7 +2158,7 @@
         <v>4</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -2178,7 +2178,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2198,7 +2198,7 @@
         <v>4</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2218,7 +2218,7 @@
         <v>4</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -2238,7 +2238,7 @@
         <v>5</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -2258,7 +2258,7 @@
         <v>4</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2278,7 +2278,7 @@
         <v>5</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2298,7 +2298,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -2318,7 +2318,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2338,7 +2338,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2358,7 +2358,7 @@
         <v>4</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,7 +2378,7 @@
         <v>4</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2398,7 +2398,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2418,7 +2418,7 @@
         <v>4</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2438,7 +2438,7 @@
         <v>4</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2458,7 +2458,7 @@
         <v>4</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2478,7 +2478,7 @@
         <v>3</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2498,7 +2498,7 @@
         <v>4</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2518,7 +2518,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2538,7 +2538,7 @@
         <v>4</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2558,7 +2558,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2578,7 +2578,7 @@
         <v>4</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2598,7 +2598,7 @@
         <v>4</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2618,7 +2618,7 @@
         <v>4</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2638,7 +2638,7 @@
         <v>4</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2658,7 +2658,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2678,7 +2678,7 @@
         <v>4</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2698,7 +2698,7 @@
         <v>4</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2718,7 +2718,7 @@
         <v>3</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2738,7 +2738,7 @@
         <v>3</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2758,7 +2758,7 @@
         <v>3</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2778,7 +2778,7 @@
         <v>3</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2798,7 +2798,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2818,7 +2818,7 @@
         <v>3</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2838,7 +2838,7 @@
         <v>4</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2858,7 +2858,7 @@
         <v>4</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2878,7 +2878,7 @@
         <v>5</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2898,7 +2898,7 @@
         <v>5</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2918,7 +2918,7 @@
         <v>4</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2938,7 +2938,7 @@
         <v>4</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2958,7 +2958,7 @@
         <v>4</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3252,18 +3252,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -3274,7 +3274,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -3285,7 +3285,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
@@ -3296,7 +3296,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
@@ -3307,7 +3307,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B7" s="1">
         <v>3</v>
@@ -3329,7 +3329,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
@@ -3512,7 +3512,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>204</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>96</v>
@@ -3520,15 +3520,15 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B7" s="1">
         <v>2</v>
@@ -3536,7 +3536,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
@@ -3544,7 +3544,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>7</v>
@@ -3552,15 +3552,15 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B11" s="1">
         <v>1</v>
@@ -3568,7 +3568,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B12" s="1">
         <v>4</v>
@@ -6906,18 +6906,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" t="s">
         <v>152</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>153</v>
-      </c>
-      <c r="C1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
         <v>84</v>
@@ -6928,7 +6928,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B3" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Sprint 4.0 - refatora schedule para aulas individuais e integra professores na exportação
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67659373-BBB2-4118-B6E4-D0D0241B1A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0156FBE-E6BF-4575-AA50-DCC27360FEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="206">
   <si>
     <t>Turma</t>
   </si>
@@ -652,6 +652,9 @@
   </si>
   <si>
     <t>CNST_COMPLEMENTO</t>
+  </si>
+  <si>
+    <t>POR_DIAS_DIFERENTES</t>
   </si>
 </sst>
 </file>
@@ -3471,7 +3474,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
@@ -3574,9 +3577,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Sprint 4A - introduz infraestrutura de otimização por áreas
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0156FBE-E6BF-4575-AA50-DCC27360FEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C66088-E369-4D09-92F8-8D38BEE6C2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="209">
   <si>
     <t>Turma</t>
   </si>
@@ -655,6 +655,15 @@
   </si>
   <si>
     <t>POR_DIAS_DIFERENTES</t>
+  </si>
+  <si>
+    <t>CHSA_BLOCO_CONTINUO</t>
+  </si>
+  <si>
+    <t>CNST_BLOCO_CONTINUO</t>
+  </si>
+  <si>
+    <t>LEST_BLOCO_CONTINUO</t>
   </si>
 </sst>
 </file>
@@ -3474,7 +3483,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
@@ -3582,6 +3591,30 @@
         <v>205</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>208</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implementa BLOCO_CONTINUO_MINIMO, validação de continuidade e integração de professores
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C66088-E369-4D09-92F8-8D38BEE6C2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CBEE98-1F5D-4D03-A47C-68BB8B57F96A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1429" uniqueCount="209">
   <si>
     <t>Turma</t>
   </si>
@@ -657,13 +657,13 @@
     <t>POR_DIAS_DIFERENTES</t>
   </si>
   <si>
-    <t>CHSA_BLOCO_CONTINUO</t>
-  </si>
-  <si>
-    <t>CNST_BLOCO_CONTINUO</t>
-  </si>
-  <si>
-    <t>LEST_BLOCO_CONTINUO</t>
+    <t>CHSA_BLOCO_CONTINUO_MINIMO</t>
+  </si>
+  <si>
+    <t>CNST_BLOCO_CONTINUO_MINIMO</t>
+  </si>
+  <si>
+    <t>LEST_BLOCO_CONTINUO_MINIMO</t>
   </si>
 </sst>
 </file>
@@ -3598,24 +3598,24 @@
       <c r="A14" t="s">
         <v>206</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>7</v>
+      <c r="B14" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>207</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>7</v>
+      <c r="B15" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>208</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>7</v>
+      <c r="B16" s="1">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 4B - compactação por componentes e validações pedagógicas
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CBEE98-1F5D-4D03-A47C-68BB8B57F96A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7DD40E-F3E2-486F-8107-DA472CCD0CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1429" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="215">
   <si>
     <t>Turma</t>
   </si>
@@ -664,6 +664,24 @@
   </si>
   <si>
     <t>LEST_BLOCO_CONTINUO_MINIMO</t>
+  </si>
+  <si>
+    <t>LEST_BLOCO_OTIMO</t>
+  </si>
+  <si>
+    <t>LEST_BLOCO_ACEITAVEL</t>
+  </si>
+  <si>
+    <t>LEST_BLOCO_MINIMO</t>
+  </si>
+  <si>
+    <t>CNST_BLOCO_OTIMO</t>
+  </si>
+  <si>
+    <t>CNST_BLOCO_MINIMO</t>
+  </si>
+  <si>
+    <t>FTP_DIAS_DIFERENTES</t>
   </si>
 </sst>
 </file>
@@ -3483,7 +3501,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
@@ -3500,87 +3518,87 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B2" s="1">
-        <v>6</v>
+        <v>204</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" s="1">
-        <v>5</v>
+        <v>142</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B4" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>204</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>96</v>
+        <v>145</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>143</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="1">
-        <v>2</v>
+        <v>214</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="1">
-        <v>2</v>
+        <v>147</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>146</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>7</v>
+        <v>149</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
+      </c>
+      <c r="B10" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>149</v>
-      </c>
-      <c r="B11" s="1">
-        <v>1</v>
+        <v>205</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>206</v>
       </c>
       <c r="B12" s="1">
         <v>4</v>
@@ -3588,15 +3606,15 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>205</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>7</v>
+        <v>207</v>
+      </c>
+      <c r="B13" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B14" s="1">
         <v>4</v>
@@ -3604,17 +3622,65 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>139</v>
       </c>
       <c r="B15" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>208</v>
+        <v>140</v>
       </c>
       <c r="B16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B19" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>212</v>
+      </c>
+      <c r="B21" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" s="1">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implementa restrição hard de disponibilidade docente e corrige loader
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,27 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77FC7954-9110-4E3D-A950-41185C44E1CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7998B49-F15A-4E25-A3C3-AE4BB745A6C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
-    <sheet name="TURMAS" sheetId="1" r:id="rId2"/>
-    <sheet name="PROFESSORES" sheetId="2" r:id="rId3"/>
-    <sheet name="ESPECIALIDADES_1ANO" sheetId="3" r:id="rId4"/>
-    <sheet name="PESOS" sheetId="12" r:id="rId5"/>
-    <sheet name="CURSOS" sheetId="4" r:id="rId6"/>
-    <sheet name="RESTRICOES" sheetId="14" r:id="rId7"/>
-    <sheet name="ATRIBUICOES" sheetId="6" r:id="rId8"/>
-    <sheet name="PARES_PEDAGOGICOS" sheetId="7" r:id="rId9"/>
-    <sheet name="PADROES_PEDAGOGICOS" sheetId="8" r:id="rId10"/>
-    <sheet name="SLOTS" sheetId="9" r:id="rId11"/>
-    <sheet name="AREAS" sheetId="10" r:id="rId12"/>
-    <sheet name="AFINIDADE_AREAS" sheetId="13" r:id="rId13"/>
+    <sheet name="DISPONIBILIDADE" sheetId="15" r:id="rId2"/>
+    <sheet name="TURMAS" sheetId="1" r:id="rId3"/>
+    <sheet name="PROFESSORES" sheetId="2" r:id="rId4"/>
+    <sheet name="ESPECIALIDADES_1ANO" sheetId="3" r:id="rId5"/>
+    <sheet name="PESOS" sheetId="12" r:id="rId6"/>
+    <sheet name="CURSOS" sheetId="4" r:id="rId7"/>
+    <sheet name="RESTRICOES" sheetId="14" r:id="rId8"/>
+    <sheet name="ATRIBUICOES" sheetId="6" r:id="rId9"/>
+    <sheet name="PARES_PEDAGOGICOS" sheetId="7" r:id="rId10"/>
+    <sheet name="PADROES_PEDAGOGICOS" sheetId="8" r:id="rId11"/>
+    <sheet name="SLOTS" sheetId="9" r:id="rId12"/>
+    <sheet name="AREAS" sheetId="10" r:id="rId13"/>
+    <sheet name="AFINIDADE_AREAS" sheetId="13" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">ATRIBUICOES!$A$1:$C$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">ATRIBUICOES!$A$1:$C$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AE$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1534" uniqueCount="243">
   <si>
     <t>Turma</t>
   </si>
@@ -687,16 +689,115 @@
   </si>
   <si>
     <t>Artes</t>
+  </si>
+  <si>
+    <t>SEG 1</t>
+  </si>
+  <si>
+    <t>SEG 2</t>
+  </si>
+  <si>
+    <t>SEG 3</t>
+  </si>
+  <si>
+    <t>SEG 4</t>
+  </si>
+  <si>
+    <t>SEG 5</t>
+  </si>
+  <si>
+    <t>SEG 6</t>
+  </si>
+  <si>
+    <t>TER 1</t>
+  </si>
+  <si>
+    <t>TER 2</t>
+  </si>
+  <si>
+    <t>TER 3</t>
+  </si>
+  <si>
+    <t>TER 4</t>
+  </si>
+  <si>
+    <t>TER 5</t>
+  </si>
+  <si>
+    <t>TER 6</t>
+  </si>
+  <si>
+    <t>QUA 1</t>
+  </si>
+  <si>
+    <t>QUA 2</t>
+  </si>
+  <si>
+    <t>QUA 3</t>
+  </si>
+  <si>
+    <t>QUA 4</t>
+  </si>
+  <si>
+    <t>QUA 5</t>
+  </si>
+  <si>
+    <t>QUA 6</t>
+  </si>
+  <si>
+    <t>QUI 1</t>
+  </si>
+  <si>
+    <t>QUI 2</t>
+  </si>
+  <si>
+    <t>QUI 3</t>
+  </si>
+  <si>
+    <t>QUI 4</t>
+  </si>
+  <si>
+    <t>QUI 5</t>
+  </si>
+  <si>
+    <t>QUI 6</t>
+  </si>
+  <si>
+    <t>SEX 1</t>
+  </si>
+  <si>
+    <t>SEX 2</t>
+  </si>
+  <si>
+    <t>SEX 3</t>
+  </si>
+  <si>
+    <t>SEX 4</t>
+  </si>
+  <si>
+    <t>SEX 5</t>
+  </si>
+  <si>
+    <t>SEX 6</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
@@ -940,7 +1041,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="1">
-        <v>1800</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -980,7 +1081,7 @@
         <v>182</v>
       </c>
       <c r="B7" s="1">
-        <v>100</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -988,7 +1089,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="1">
-        <v>80</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -996,7 +1097,7 @@
         <v>184</v>
       </c>
       <c r="B9" s="1">
-        <v>60</v>
+        <v>2500</v>
       </c>
     </row>
   </sheetData>
@@ -1005,6 +1106,53 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1152,7 +1300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1414,7 +1562,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1485,7 +1633,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42872D3-F405-45C3-ACE9-05765074B023}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1573,6 +1721,435 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A23CC3-1A6A-46FD-BA52-7A9B0C051B2C}">
+  <dimension ref="A1:AE53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="31" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AE53" xr:uid="{59A23CC3-1A6A-46FD-BA52-7A9B0C051B2C}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE53">
+      <sortCondition ref="A1:A53"/>
+    </sortState>
+  </autoFilter>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1924,7 +2501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F53"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3002,7 +3579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3275,7 +3852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F3F9048-A942-472C-8750-2838F0F7C4D7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3389,7 +3966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3504,7 +4081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{630F621C-FE58-421F-BCF4-47DF583B060A}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3671,7 +4248,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C300"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6985,51 +7562,4 @@
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="3" width="17.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: injeção automática de PA/PV e criação do Dashboard de Qualidade
- Implementado Dashboard no ExcelExporter com tempo de execução e medidor de fragmentação.
- Correção de tipagem (float/nan) do Pandas ao ler 'Anos_atuacao'.
- Injeção inteligente de PA e PV na grade dos professores nos espaços livres.
- Correção do identificador de turma virtual para evitar sobrescrita de slots de projetos.
- ExcelExporter configurado para exibir apenas o texto limpo ('PA' ou 'PV') nos blocos de PROJETO.
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA559E00-77BF-463A-BF6C-1765F0127DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F9319B-BF00-407A-9EFF-6E2ACE5B2AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -33,7 +33,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">ATRIBUICOES!$A$1:$C$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AE$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">PROFESSORES!$A$1:$H$788</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">PROFESSORES!$A$1:$H$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TURMAS!$A$1:$E$70</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4471" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4485" uniqueCount="437">
   <si>
     <t>Turma</t>
   </si>
@@ -1347,6 +1347,27 @@
   </si>
   <si>
     <t>Negócios</t>
+  </si>
+  <si>
+    <t>PLAN LEST</t>
+  </si>
+  <si>
+    <t>PLAN MEST</t>
+  </si>
+  <si>
+    <t>PLAN CNST</t>
+  </si>
+  <si>
+    <t>PLAN CHSA</t>
+  </si>
+  <si>
+    <t>PLAN FTP TEC</t>
+  </si>
+  <si>
+    <t>PLAN FTP NEG</t>
+  </si>
+  <si>
+    <t>PLAN FTP MMD</t>
   </si>
 </sst>
 </file>
@@ -1606,7 +1627,7 @@
         <v>114</v>
       </c>
       <c r="B2" s="1">
-        <v>300</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -14173,10 +14194,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>225</v>
+        <v>44</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>7</v>
@@ -14190,10 +14211,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>225</v>
+        <v>44</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>7</v>
@@ -15271,7 +15292,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1">
         <v>3</v>
@@ -15369,7 +15390,7 @@
         <v>38</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1">
         <v>1</v>
@@ -15484,7 +15505,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D13" s="1">
         <v>2</v>
@@ -15530,7 +15551,7 @@
         <v>36</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D15" s="1">
         <v>2</v>
@@ -15648,7 +15669,7 @@
         <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D20" s="1">
         <v>2</v>
@@ -15786,7 +15807,7 @@
         <v>37</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D26" s="1">
         <v>1</v>
@@ -15999,7 +16020,7 @@
         <v>36</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D35" s="1">
         <v>2</v>
@@ -16097,7 +16118,7 @@
         <v>34</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D39" s="1">
         <v>3</v>
@@ -16120,7 +16141,7 @@
         <v>36</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D40" s="1">
         <v>1</v>
@@ -16192,7 +16213,7 @@
         <v>37</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D43" s="1">
         <v>3</v>
@@ -16523,7 +16544,7 @@
         <v>37</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D57" s="1">
         <v>2</v>
@@ -16618,7 +16639,7 @@
         <v>37</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D61" s="1">
         <v>2</v>
@@ -16687,7 +16708,7 @@
         <v>36</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D64" s="1">
         <v>1</v>
@@ -16733,7 +16754,7 @@
         <v>38</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D66" s="1">
         <v>2</v>
@@ -16779,7 +16800,7 @@
         <v>38</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D68" s="1">
         <v>3</v>
@@ -16943,7 +16964,7 @@
         <v>34</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D75" s="1">
         <v>1</v>
@@ -17035,7 +17056,7 @@
         <v>34</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D79" s="1">
         <v>1</v>
@@ -17127,7 +17148,7 @@
         <v>37</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D83" s="1">
         <v>3</v>
@@ -17173,7 +17194,7 @@
         <v>36</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D85" s="1">
         <v>3</v>
@@ -17196,7 +17217,7 @@
         <v>37</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D86" s="1">
         <v>3</v>
@@ -17245,7 +17266,7 @@
         <v>36</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D88" s="1">
         <v>1</v>
@@ -17268,7 +17289,7 @@
         <v>34</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D89" s="1">
         <v>2</v>
@@ -17340,7 +17361,7 @@
         <v>34</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D92" s="1">
         <v>3</v>
@@ -17481,7 +17502,7 @@
         <v>38</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D98" s="1">
         <v>2</v>
@@ -17504,7 +17525,7 @@
         <v>38</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D99" s="1">
         <v>3</v>
@@ -17573,7 +17594,7 @@
         <v>38</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D102" s="1">
         <v>1</v>
@@ -17740,7 +17761,7 @@
         <v>37</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D109" s="1">
         <v>1</v>
@@ -17809,7 +17830,7 @@
         <v>34</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D112" s="1">
         <v>1</v>
@@ -17901,7 +17922,7 @@
         <v>37</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D116" s="1">
         <v>1</v>
@@ -17924,7 +17945,7 @@
         <v>36</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D117" s="1">
         <v>1</v>
@@ -18016,7 +18037,7 @@
         <v>37</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D121" s="1">
         <v>2</v>
@@ -18039,7 +18060,7 @@
         <v>38</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D122" s="1">
         <v>2</v>
@@ -18249,7 +18270,7 @@
         <v>38</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D131" s="1">
         <v>3</v>
@@ -18295,7 +18316,7 @@
         <v>37</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D133" s="1">
         <v>2</v>
@@ -18367,7 +18388,7 @@
         <v>34</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D136" s="1">
         <v>1</v>
@@ -18485,7 +18506,7 @@
         <v>36</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D141" s="1">
         <v>3</v>
@@ -18721,7 +18742,7 @@
         <v>34</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D151" s="1">
         <v>3</v>
@@ -20774,6 +20795,7 @@
       <c r="H788" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H157" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -21720,7 +21742,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -21750,9 +21772,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="str">
-        <f>"PLAN "&amp;E2</f>
-        <v>PLAN LEST</v>
+      <c r="A2" t="s">
+        <v>430</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -21765,9 +21786,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="str">
-        <f t="shared" ref="A3:A6" si="0">"PLAN "&amp;E3</f>
-        <v>PLAN MEST</v>
+      <c r="A3" t="s">
+        <v>431</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -21780,9 +21800,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="str">
-        <f t="shared" si="0"/>
-        <v>PLAN CNST</v>
+      <c r="A4" t="s">
+        <v>432</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
@@ -21795,9 +21814,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="str">
-        <f t="shared" si="0"/>
-        <v>PLAN CHSA</v>
+      <c r="A5" t="s">
+        <v>433</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
@@ -21810,9 +21828,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="str">
-        <f t="shared" si="0"/>
-        <v>PLAN FTP</v>
+      <c r="A6" t="s">
+        <v>434</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
@@ -21820,7 +21837,44 @@
       <c r="C6" s="1" t="s">
         <v>258</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="E6" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>435</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>436</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>43</v>
       </c>
     </row>
@@ -21828,7 +21882,7 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="C4:C6 C2:C3" twoDigitTextYear="1"/>
+    <ignoredError sqref="C4:C6 C2:C3 C7:C8" twoDigitTextYear="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Inclusão de atividades avulsas definidas na planilha de geração do horário
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B23DF7-78DB-4B44-8A12-63A214CB3866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF7B2E3-45FA-459B-945A-2115D6ACAAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,12 @@
     <sheet name="TURMAS" sheetId="1" r:id="rId3"/>
     <sheet name="PROFESSORES" sheetId="2" r:id="rId4"/>
     <sheet name="ATRIBUICOES" sheetId="6" r:id="rId5"/>
-    <sheet name="ESPECIALIDADES" sheetId="3" r:id="rId6"/>
-    <sheet name="PLANEJAMENTO" sheetId="16" r:id="rId7"/>
-    <sheet name="PESOS" sheetId="12" r:id="rId8"/>
-    <sheet name="CURSOS" sheetId="4" r:id="rId9"/>
-    <sheet name="RESTRICOES" sheetId="14" r:id="rId10"/>
-    <sheet name="ATIVIDADES_AVULSAS" sheetId="17" r:id="rId11"/>
+    <sheet name="ATIVIDADES_AVULSAS" sheetId="17" r:id="rId6"/>
+    <sheet name="ESPECIALIDADES" sheetId="3" r:id="rId7"/>
+    <sheet name="PLANEJAMENTO" sheetId="16" r:id="rId8"/>
+    <sheet name="PESOS" sheetId="12" r:id="rId9"/>
+    <sheet name="CURSOS" sheetId="4" r:id="rId10"/>
+    <sheet name="RESTRICOES" sheetId="14" r:id="rId11"/>
     <sheet name="PARES_PEDAGOGICOS" sheetId="7" r:id="rId12"/>
     <sheet name="PADROES_PEDAGOGICOS" sheetId="8" r:id="rId13"/>
     <sheet name="SLOTS" sheetId="9" r:id="rId14"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4486" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4499" uniqueCount="439">
   <si>
     <t>Turma</t>
   </si>
@@ -1371,6 +1371,9 @@
   </si>
   <si>
     <t>Plan_Ind</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -1630,8 +1633,7 @@
         <v>114</v>
       </c>
       <c r="B2" s="1">
-        <f>3*60</f>
-        <v>180</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1696,6 +1698,163 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B8" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B9" t="s">
+        <v>224</v>
+      </c>
+      <c r="C9" t="s">
+        <v>224</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>255</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{630F621C-FE58-421F-BCF4-47DF583B060A}">
   <dimension ref="A1:B34"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1979,74 +2138,6 @@
   </sheetData>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D90FE78-749D-4E79-8923-ED8BD0B01BA1}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1"/>
-    <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
-        <v>260</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>300</v>
-      </c>
-      <c r="B2" t="s">
-        <v>262</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D2" s="1">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>268</v>
-      </c>
-      <c r="B3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
@@ -2743,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A23CC3-1A6A-46FD-BA52-7A9B0C051B2C}">
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
@@ -2843,6 +2934,49 @@
       </c>
       <c r="AE1" s="1" t="s">
         <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>398</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>359</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>438</v>
       </c>
     </row>
   </sheetData>
@@ -21566,6 +21700,74 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D90FE78-749D-4E79-8923-ED8BD0B01BA1}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -22683,7 +22885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -22830,7 +23032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F3F9048-A942-472C-8750-2838F0F7C4D7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -22942,161 +23144,4 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="8.28515625" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>253</v>
-      </c>
-      <c r="B8" t="s">
-        <v>225</v>
-      </c>
-      <c r="C8" t="s">
-        <v>225</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>254</v>
-      </c>
-      <c r="B9" t="s">
-        <v>224</v>
-      </c>
-      <c r="C9" t="s">
-        <v>224</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>255</v>
-      </c>
-      <c r="B10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correção da imposição de dias máximos para cada professor.
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF7B2E3-45FA-459B-945A-2115D6ACAAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4591753-DB3F-4D10-82C9-C6099959ADE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -4315,7 +4315,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>131</v>
@@ -4399,7 +4399,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>131</v>
@@ -4459,7 +4459,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>45</v>
@@ -4471,10 +4471,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G10" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H10" s="1">
         <v>5</v>
@@ -4485,10 +4485,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>46</v>
@@ -4497,13 +4497,13 @@
         <v>3</v>
       </c>
       <c r="F11" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G11" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H11" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>131</v>
@@ -4511,25 +4511,25 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D12" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G12" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H12" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>131</v>
@@ -4537,25 +4537,25 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D13" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G13" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H13" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>131</v>
@@ -4563,13 +4563,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D14" s="1">
         <v>2</v>
@@ -4578,7 +4578,7 @@
         <v>30</v>
       </c>
       <c r="G14" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H14" s="1">
         <v>5</v>
@@ -4589,22 +4589,22 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D15" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="1">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G15" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H15" s="1">
         <v>5</v>
@@ -4615,25 +4615,28 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D16" s="1">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F16" s="1">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G16" s="1">
+        <v>5</v>
+      </c>
+      <c r="H16" s="1">
         <v>4</v>
-      </c>
-      <c r="H16" s="1">
-        <v>5</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>131</v>
@@ -4641,25 +4644,25 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D17" s="1">
         <v>2</v>
       </c>
       <c r="F17" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G17" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H17" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>131</v>
@@ -4667,22 +4670,22 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G18" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H18" s="1">
         <v>5</v>
@@ -4693,25 +4696,22 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D19" s="1">
         <v>2</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F19" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G19" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H19" s="1">
         <v>5</v>
@@ -4722,19 +4722,19 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D20" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G20" s="1">
         <v>8</v>
@@ -4748,13 +4748,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D21" s="1">
         <v>3</v>
@@ -4763,7 +4763,7 @@
         <v>30</v>
       </c>
       <c r="G21" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H21" s="1">
         <v>5</v>
@@ -4774,22 +4774,22 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D22" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G22" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H22" s="1">
         <v>5</v>
@@ -4800,22 +4800,22 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D23" s="1">
         <v>1</v>
       </c>
       <c r="F23" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G23" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H23" s="1">
         <v>5</v>
@@ -4826,16 +4826,16 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D24" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" s="1">
         <v>30</v>
@@ -4852,25 +4852,28 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D25" s="1">
         <v>1</v>
       </c>
+      <c r="E25" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="F25" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G25" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H25" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>131</v>
@@ -4878,25 +4881,25 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D26" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G26" s="1">
         <v>4</v>
       </c>
       <c r="H26" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>131</v>
@@ -4904,25 +4907,28 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D27" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="F27" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G27" s="1">
         <v>5</v>
       </c>
       <c r="H27" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>131</v>
@@ -4930,25 +4936,22 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D28" s="1">
-        <v>1</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="F28" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G28" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H28" s="1">
         <v>5</v>
@@ -4959,25 +4962,25 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D29" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" s="1">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G29" s="1">
+        <v>8</v>
+      </c>
+      <c r="H29" s="1">
         <v>4</v>
-      </c>
-      <c r="H29" s="1">
-        <v>5</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>131</v>
@@ -4985,20 +4988,17 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>429</v>
-      </c>
       <c r="F30" s="1">
         <v>24</v>
       </c>
@@ -5006,7 +5006,7 @@
         <v>5</v>
       </c>
       <c r="H30" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>131</v>
@@ -5014,10 +5014,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>40</v>
@@ -5026,13 +5026,13 @@
         <v>2</v>
       </c>
       <c r="F31" s="1">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G31" s="1">
         <v>6</v>
       </c>
       <c r="H31" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>131</v>
@@ -5040,19 +5040,19 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D32" s="1">
         <v>2</v>
       </c>
       <c r="F32" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G32" s="1">
         <v>8</v>
@@ -5066,19 +5066,22 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D33" s="1">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="F33" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G33" s="1">
         <v>5</v>
@@ -5092,25 +5095,28 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D34" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F34" s="1">
         <v>22</v>
       </c>
       <c r="G34" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H34" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>131</v>
@@ -5118,22 +5124,22 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D35" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" s="1">
         <v>26</v>
       </c>
       <c r="G35" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H35" s="1">
         <v>5</v>
@@ -5144,25 +5150,22 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D36" s="1">
-        <v>2</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>429</v>
+        <v>3</v>
       </c>
       <c r="F36" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G36" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H36" s="1">
         <v>5</v>
@@ -5173,7 +5176,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>43</v>
@@ -5185,16 +5188,16 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>110</v>
+        <v>71</v>
       </c>
       <c r="F37" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G37" s="1">
         <v>5</v>
       </c>
       <c r="H37" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>131</v>
@@ -5202,25 +5205,25 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="F38" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G38" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H38" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>131</v>
@@ -5228,22 +5231,22 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D39" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F39" s="1">
         <v>30</v>
       </c>
       <c r="G39" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H39" s="1">
         <v>5</v>
@@ -5254,22 +5257,25 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D40" s="1">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F40" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G40" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H40" s="1">
         <v>5</v>
@@ -5280,22 +5286,22 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D41" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F41" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G41" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H41" s="1">
         <v>5</v>
@@ -5306,25 +5312,22 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D42" s="1">
-        <v>2</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>110</v>
+        <v>3</v>
       </c>
       <c r="F42" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G42" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H42" s="1">
         <v>5</v>
@@ -5335,22 +5338,22 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D43" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" s="1">
         <v>26</v>
       </c>
       <c r="G43" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H43" s="1">
         <v>5</v>
@@ -5361,22 +5364,19 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>315</v>
+        <v>276</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D44" s="1">
-        <v>1</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="F44" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G44" s="1">
         <v>5</v>
@@ -5390,22 +5390,22 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D45" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F45" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G45" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H45" s="1">
         <v>5</v>
@@ -5416,22 +5416,22 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D46" s="1">
         <v>2</v>
       </c>
       <c r="F46" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G46" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H46" s="1">
         <v>5</v>
@@ -5442,7 +5442,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>41</v>
@@ -5468,10 +5468,10 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>46</v>
@@ -5483,7 +5483,7 @@
         <v>26</v>
       </c>
       <c r="G48" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H48" s="1">
         <v>5</v>
@@ -5494,22 +5494,22 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D49" s="1">
         <v>2</v>
       </c>
       <c r="F49" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G49" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H49" s="1">
         <v>5</v>
@@ -5520,10 +5520,10 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>40</v>
@@ -5532,13 +5532,13 @@
         <v>1</v>
       </c>
       <c r="F50" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G50" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H50" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>131</v>
@@ -5546,22 +5546,25 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D51" s="1">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F51" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G51" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H51" s="1">
         <v>5</v>
@@ -5572,7 +5575,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>49</v>
@@ -5581,10 +5584,10 @@
         <v>46</v>
       </c>
       <c r="D52" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G52" s="1">
         <v>5</v>
@@ -5598,22 +5601,25 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D53" s="1">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F53" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G53" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H53" s="1">
         <v>5</v>
@@ -5624,7 +5630,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>43</v>
@@ -5633,16 +5639,16 @@
         <v>43</v>
       </c>
       <c r="D54" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>110</v>
+        <v>71</v>
       </c>
       <c r="F54" s="1">
         <v>30</v>
       </c>
       <c r="G54" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H54" s="1">
         <v>5</v>
@@ -5653,25 +5659,25 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D55" s="1">
         <v>3</v>
       </c>
       <c r="F55" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G55" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H55" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>131</v>
@@ -5679,19 +5685,16 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D56" s="1">
-        <v>3</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>110</v>
+        <v>1</v>
       </c>
       <c r="F56" s="1">
         <v>30</v>
@@ -5708,7 +5711,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>37</v>
@@ -5720,7 +5723,7 @@
         <v>2</v>
       </c>
       <c r="F57" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G57" s="1">
         <v>5</v>
@@ -5734,25 +5737,22 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="D58" s="1">
-        <v>3</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="F58" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G58" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H58" s="1">
         <v>5</v>
@@ -5763,25 +5763,25 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D59" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F59" s="1">
         <v>24</v>
       </c>
       <c r="G59" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H59" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>131</v>
@@ -5789,7 +5789,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>47</v>
@@ -5801,7 +5801,7 @@
         <v>1</v>
       </c>
       <c r="F60" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G60" s="1">
         <v>5</v>
@@ -5815,10 +5815,10 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>35</v>
@@ -5841,25 +5841,25 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D62" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G62" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H62" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>131</v>
@@ -5867,19 +5867,19 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D63" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F63" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G63" s="1">
         <v>5</v>
@@ -5893,19 +5893,19 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D64" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F64" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G64" s="1">
         <v>5</v>
@@ -5919,13 +5919,13 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D65" s="1">
         <v>1</v>
@@ -5945,13 +5945,13 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D66" s="1">
         <v>2</v>
@@ -5971,22 +5971,22 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D67" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F67" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G67" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H67" s="1">
         <v>5</v>
@@ -5997,19 +5997,22 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D68" s="1">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="F68" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G68" s="1">
         <v>5</v>
@@ -6023,25 +6026,25 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D69" s="1">
         <v>3</v>
       </c>
       <c r="F69" s="1">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G69" s="1">
         <v>5</v>
       </c>
       <c r="H69" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>131</v>
@@ -6049,13 +6052,13 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D70" s="1">
         <v>1</v>
@@ -6075,7 +6078,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>48</v>
@@ -6084,13 +6087,13 @@
         <v>46</v>
       </c>
       <c r="D71" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G71" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H71" s="1">
         <v>5</v>
@@ -6101,28 +6104,25 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D72" s="1">
-        <v>1</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>429</v>
+        <v>3</v>
       </c>
       <c r="F72" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G72" s="1">
         <v>5</v>
       </c>
       <c r="H72" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I72" s="1" t="s">
         <v>131</v>
@@ -6130,22 +6130,22 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D73" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F73" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G73" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H73" s="1">
         <v>5</v>
@@ -6156,25 +6156,25 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D74" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F74" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G74" s="1">
         <v>5</v>
       </c>
       <c r="H74" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I74" s="1" t="s">
         <v>131</v>
@@ -6182,13 +6182,13 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D75" s="1">
         <v>1</v>
@@ -6197,7 +6197,7 @@
         <v>26</v>
       </c>
       <c r="G75" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H75" s="1">
         <v>5</v>
@@ -6208,19 +6208,19 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D76" s="1">
         <v>1</v>
       </c>
       <c r="F76" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G76" s="1">
         <v>6</v>
@@ -6234,7 +6234,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>39</v>
@@ -6243,16 +6243,16 @@
         <v>40</v>
       </c>
       <c r="D77" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F77" s="1">
         <v>24</v>
       </c>
       <c r="G77" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H77" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I77" s="1" t="s">
         <v>131</v>
@@ -6260,22 +6260,22 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D78" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78" s="1">
         <v>26</v>
       </c>
       <c r="G78" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H78" s="1">
         <v>5</v>
@@ -6286,25 +6286,25 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D79" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F79" s="1">
         <v>24</v>
       </c>
       <c r="G79" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H79" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>131</v>
@@ -6312,16 +6312,16 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D80" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80" s="1">
         <v>26</v>
@@ -6338,16 +6338,16 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D81" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F81" s="1">
         <v>26</v>
@@ -6364,25 +6364,28 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D82" s="1">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F82" s="1">
         <v>24</v>
       </c>
       <c r="G82" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H82" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I82" s="1" t="s">
         <v>131</v>
@@ -6390,22 +6393,22 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D83" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F83" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G83" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H83" s="1">
         <v>5</v>
@@ -6416,22 +6419,22 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D84" s="1">
         <v>2</v>
       </c>
       <c r="F84" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G84" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H84" s="1">
         <v>5</v>
@@ -6442,22 +6445,22 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D85" s="1">
         <v>3</v>
       </c>
       <c r="F85" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G85" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H85" s="1">
         <v>5</v>
@@ -6468,22 +6471,25 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D86" s="1">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F86" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G86" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H86" s="1">
         <v>5</v>
@@ -6494,25 +6500,22 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D87" s="1">
         <v>3</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F87" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G87" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H87" s="1">
         <v>5</v>
@@ -6523,19 +6526,19 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D88" s="1">
         <v>1</v>
       </c>
       <c r="F88" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G88" s="1">
         <v>5</v>
@@ -6549,22 +6552,22 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D89" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F89" s="1">
         <v>30</v>
       </c>
       <c r="G89" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H89" s="1">
         <v>5</v>
@@ -6575,22 +6578,25 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D90" s="1">
         <v>3</v>
       </c>
+      <c r="E90" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="F90" s="1">
         <v>26</v>
       </c>
       <c r="G90" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H90" s="1">
         <v>5</v>
@@ -6601,25 +6607,22 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D91" s="1">
-        <v>1</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="F91" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G91" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H91" s="1">
         <v>5</v>
@@ -6630,22 +6633,22 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D92" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" s="1">
         <v>30</v>
       </c>
       <c r="G92" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H92" s="1">
         <v>5</v>
@@ -6656,25 +6659,25 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D93" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F93" s="1">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="G93" s="1">
         <v>5</v>
       </c>
       <c r="H93" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I93" s="1" t="s">
         <v>131</v>
@@ -6682,13 +6685,13 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D94" s="1">
         <v>3</v>
@@ -6708,22 +6711,22 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D95" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" s="1">
         <v>26</v>
       </c>
       <c r="G95" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H95" s="1">
         <v>5</v>
@@ -6734,25 +6737,22 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>367</v>
+        <v>328</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D96" s="1">
-        <v>3</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="F96" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G96" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H96" s="1">
         <v>5</v>
@@ -6763,13 +6763,13 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D97" s="1">
         <v>2</v>
@@ -6778,7 +6778,7 @@
         <v>30</v>
       </c>
       <c r="G97" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H97" s="1">
         <v>5</v>
@@ -6789,7 +6789,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>38</v>
@@ -6798,13 +6798,13 @@
         <v>35</v>
       </c>
       <c r="D98" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" s="1">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G98" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H98" s="1">
         <v>5</v>
@@ -6815,16 +6815,19 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D99" s="1">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F99" s="1">
         <v>30</v>
@@ -6841,22 +6844,22 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D100" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F100" s="1">
         <v>26</v>
       </c>
       <c r="G100" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H100" s="1">
         <v>5</v>
@@ -6867,22 +6870,22 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D101" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F101" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G101" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H101" s="1">
         <v>5</v>
@@ -6893,22 +6896,22 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D102" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" s="1">
         <v>30</v>
       </c>
       <c r="G102" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H102" s="1">
         <v>5</v>
@@ -6919,20 +6922,17 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D103" s="1">
         <v>1</v>
       </c>
-      <c r="E103" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="F103" s="1">
         <v>30</v>
       </c>
@@ -6948,22 +6948,25 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D104" s="1">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F104" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G104" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H104" s="1">
         <v>5</v>
@@ -6974,22 +6977,22 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D105" s="1">
         <v>1</v>
       </c>
       <c r="F105" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G105" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H105" s="1">
         <v>5</v>
@@ -7000,13 +7003,13 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>377</v>
+        <v>282</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D106" s="1">
         <v>2</v>
@@ -7026,19 +7029,19 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D107" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F107" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G107" s="1">
         <v>5</v>
@@ -7052,25 +7055,22 @@
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D108" s="1">
         <v>2</v>
       </c>
-      <c r="E108" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F108" s="1">
         <v>30</v>
       </c>
       <c r="G108" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H108" s="1">
         <v>5</v>
@@ -7081,10 +7081,10 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>35</v>
@@ -7096,7 +7096,7 @@
         <v>30</v>
       </c>
       <c r="G109" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H109" s="1">
         <v>5</v>
@@ -7107,13 +7107,13 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>381</v>
+        <v>392</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D110" s="1">
         <v>2</v>
@@ -7133,19 +7133,19 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D111" s="1">
         <v>2</v>
       </c>
       <c r="F111" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G111" s="1">
         <v>5</v>
@@ -7159,22 +7159,22 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D112" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F112" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H112" s="1">
         <v>5</v>
@@ -7281,7 +7281,7 @@
         <v>6</v>
       </c>
       <c r="H116" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I116" s="1" t="s">
         <v>131</v>
@@ -7307,7 +7307,7 @@
         <v>5</v>
       </c>
       <c r="H117" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I117" s="1" t="s">
         <v>131</v>
@@ -7333,7 +7333,7 @@
         <v>5</v>
       </c>
       <c r="H118" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I118" s="1" t="s">
         <v>131</v>
@@ -7393,19 +7393,22 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D121" s="1">
         <v>2</v>
       </c>
+      <c r="E121" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="F121" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G121" s="1">
         <v>5</v>
@@ -7419,25 +7422,25 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D122" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F122" s="1">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H122" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I122" s="1" t="s">
         <v>131</v>
@@ -7445,7 +7448,7 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>50</v>
@@ -7454,13 +7457,13 @@
         <v>51</v>
       </c>
       <c r="D123" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F123" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H123" s="1">
         <v>5</v>
@@ -7471,25 +7474,22 @@
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D124" s="1">
-        <v>2</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>110</v>
+        <v>3</v>
       </c>
       <c r="F124" s="1">
         <v>30</v>
       </c>
       <c r="G124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H124" s="1">
         <v>5</v>
@@ -7500,10 +7500,10 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>40</v>
@@ -7512,7 +7512,7 @@
         <v>3</v>
       </c>
       <c r="F125" s="1">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G125" s="1">
         <v>5</v>
@@ -7526,25 +7526,25 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D126" s="1">
         <v>3</v>
       </c>
       <c r="F126" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G126" s="1">
+        <v>6</v>
+      </c>
+      <c r="H126" s="1">
         <v>4</v>
-      </c>
-      <c r="H126" s="1">
-        <v>5</v>
       </c>
       <c r="I126" s="1" t="s">
         <v>131</v>
@@ -7552,25 +7552,25 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D127" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F127" s="1">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H127" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I127" s="1" t="s">
         <v>131</v>
@@ -7578,19 +7578,19 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D128" s="1">
         <v>3</v>
       </c>
       <c r="F128" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G128" s="1">
         <v>5</v>
@@ -7604,22 +7604,22 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>400</v>
+        <v>283</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D129" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F129" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G129" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H129" s="1">
         <v>5</v>
@@ -7630,25 +7630,25 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D130" s="1">
         <v>2</v>
       </c>
       <c r="F130" s="1">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G130" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H130" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I130" s="1" t="s">
         <v>131</v>
@@ -7656,16 +7656,16 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D131" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F131" s="1">
         <v>26</v>
@@ -7682,22 +7682,22 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D132" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F132" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G132" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H132" s="1">
         <v>5</v>
@@ -7708,19 +7708,22 @@
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D133" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="F133" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G133" s="1">
         <v>5</v>
@@ -7734,19 +7737,19 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D134" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F134" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G134" s="1">
         <v>5</v>
@@ -7760,19 +7763,16 @@
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D135" s="1">
-        <v>1</v>
-      </c>
-      <c r="E135" s="1" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="F135" s="1">
         <v>30</v>
@@ -7789,22 +7789,22 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D136" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F136" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G136" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H136" s="1">
         <v>5</v>
@@ -7815,19 +7815,19 @@
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D137" s="1">
         <v>2</v>
       </c>
       <c r="F137" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G137" s="1">
         <v>5</v>
@@ -7841,22 +7841,25 @@
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D138" s="1">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="F138" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G138" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H138" s="1">
         <v>5</v>
@@ -7867,22 +7870,22 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D139" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F139" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G139" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H139" s="1">
         <v>5</v>
@@ -7893,22 +7896,19 @@
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D140" s="1">
-        <v>3</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>429</v>
+        <v>1</v>
       </c>
       <c r="F140" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G140" s="1">
         <v>5</v>
@@ -7922,25 +7922,25 @@
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D141" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F141" s="1">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G141" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H141" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I141" s="1" t="s">
         <v>131</v>
@@ -7948,19 +7948,19 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D142" s="1">
         <v>1</v>
       </c>
       <c r="F142" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G142" s="1">
         <v>5</v>
@@ -7974,19 +7974,19 @@
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D143" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F143" s="1">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G143" s="1">
         <v>5</v>
@@ -8000,7 +8000,7 @@
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>50</v>
@@ -8009,13 +8009,13 @@
         <v>51</v>
       </c>
       <c r="D144" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="1">
         <v>30</v>
       </c>
       <c r="G144" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H144" s="1">
         <v>5</v>
@@ -8026,16 +8026,16 @@
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D145" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F145" s="1">
         <v>26</v>
@@ -8052,25 +8052,28 @@
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D146" s="1">
         <v>2</v>
       </c>
+      <c r="E146" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="F146" s="1">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G146" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H146" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I146" s="1" t="s">
         <v>131</v>
@@ -8078,25 +8081,28 @@
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D147" s="1">
         <v>3</v>
       </c>
+      <c r="E147" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="F147" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G147" s="1">
         <v>5</v>
       </c>
       <c r="H147" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I147" s="1" t="s">
         <v>131</v>
@@ -8104,25 +8110,22 @@
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D148" s="1">
         <v>3</v>
       </c>
-      <c r="E148" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F148" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G148" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H148" s="1">
         <v>5</v>
@@ -8133,25 +8136,25 @@
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D149" s="1">
         <v>3</v>
       </c>
       <c r="F149" s="1">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G149" s="1">
         <v>6</v>
       </c>
       <c r="H149" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I149" s="1" t="s">
         <v>131</v>
@@ -8159,22 +8162,19 @@
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>421</v>
+        <v>319</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D150" s="1">
-        <v>2</v>
-      </c>
-      <c r="E150" s="1" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="F150" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G150" s="1">
         <v>5</v>
@@ -8188,22 +8188,25 @@
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D151" s="1">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F151" s="1">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="G151" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H151" s="1">
         <v>5</v>
@@ -8214,25 +8217,22 @@
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D152" s="1">
         <v>1</v>
       </c>
-      <c r="E152" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F152" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G152" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H152" s="1">
         <v>5</v>
@@ -8243,22 +8243,22 @@
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D153" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F153" s="1">
         <v>26</v>
       </c>
       <c r="G153" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H153" s="1">
         <v>5</v>
@@ -8269,25 +8269,25 @@
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D154" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F154" s="1">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G154" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H154" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I154" s="1" t="s">
         <v>131</v>
@@ -8295,25 +8295,25 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D155" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F155" s="1">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G155" s="1">
+        <v>8</v>
+      </c>
+      <c r="H155" s="1">
         <v>4</v>
-      </c>
-      <c r="H155" s="1">
-        <v>5</v>
       </c>
       <c r="I155" s="1" t="s">
         <v>131</v>
@@ -8321,25 +8321,28 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D156" s="1">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>429</v>
       </c>
       <c r="F156" s="1">
         <v>24</v>
       </c>
       <c r="G156" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H156" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I156" s="1" t="s">
         <v>131</v>
@@ -8347,22 +8350,19 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>428</v>
+        <v>334</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D157" s="1">
-        <v>3</v>
-      </c>
-      <c r="E157" s="1" t="s">
-        <v>429</v>
+        <v>2</v>
       </c>
       <c r="F157" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G157" s="1">
         <v>5</v>
@@ -10268,7 +10268,11 @@
       <c r="I788" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I157" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:I157" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I157">
+      <sortCondition ref="A1:A157"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
feat: Implementação da inserção de PLANEJAMENTo individual, sem choque, seguindo informação da planilha.
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4591753-DB3F-4D10-82C9-C6099959ADE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CCF78F-7D5C-4212-8E99-BF6A923D9655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
     <sheet name="DISPONIBILIDADE" sheetId="15" r:id="rId2"/>
     <sheet name="TURMAS" sheetId="1" r:id="rId3"/>
     <sheet name="PROFESSORES" sheetId="2" r:id="rId4"/>
-    <sheet name="ATRIBUICOES" sheetId="6" r:id="rId5"/>
-    <sheet name="ATIVIDADES_AVULSAS" sheetId="17" r:id="rId6"/>
-    <sheet name="ESPECIALIDADES" sheetId="3" r:id="rId7"/>
-    <sheet name="PLANEJAMENTO" sheetId="16" r:id="rId8"/>
+    <sheet name="PLANEJAMENTO" sheetId="16" r:id="rId5"/>
+    <sheet name="ATRIBUICOES" sheetId="6" r:id="rId6"/>
+    <sheet name="ATIVIDADES_AVULSAS" sheetId="17" r:id="rId7"/>
+    <sheet name="ESPECIALIDADES" sheetId="3" r:id="rId8"/>
     <sheet name="PESOS" sheetId="12" r:id="rId9"/>
     <sheet name="CURSOS" sheetId="4" r:id="rId10"/>
     <sheet name="RESTRICOES" sheetId="14" r:id="rId11"/>
@@ -31,7 +31,7 @@
     <sheet name="AFINIDADE_AREAS" sheetId="13" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">ATRIBUICOES!$A$1:$C$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">ATRIBUICOES!$A$1:$C$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AE$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">PROFESSORES!$A$1:$I$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TURMAS!$A$1:$E$70</definedName>
@@ -4260,7 +4260,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2" s="1">
         <v>5</v>
@@ -4286,7 +4286,7 @@
         <v>26</v>
       </c>
       <c r="G3" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H3" s="1">
         <v>5</v>
@@ -4312,7 +4312,7 @@
         <v>24</v>
       </c>
       <c r="G4" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H4" s="1">
         <v>4</v>
@@ -4341,7 +4341,7 @@
         <v>30</v>
       </c>
       <c r="G5" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H5" s="1">
         <v>5</v>
@@ -4370,7 +4370,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" s="1">
         <v>5</v>
@@ -4396,7 +4396,7 @@
         <v>24</v>
       </c>
       <c r="G7" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H7" s="1">
         <v>4</v>
@@ -4422,7 +4422,7 @@
         <v>26</v>
       </c>
       <c r="G8" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="1">
         <v>5</v>
@@ -4448,7 +4448,7 @@
         <v>26</v>
       </c>
       <c r="G9" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H9" s="1">
         <v>5</v>
@@ -4474,7 +4474,7 @@
         <v>26</v>
       </c>
       <c r="G10" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H10" s="1">
         <v>5</v>
@@ -4500,7 +4500,7 @@
         <v>24</v>
       </c>
       <c r="G11" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H11" s="1">
         <v>4</v>
@@ -4526,7 +4526,7 @@
         <v>23</v>
       </c>
       <c r="G12" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H12" s="1">
         <v>4</v>
@@ -4552,7 +4552,7 @@
         <v>20</v>
       </c>
       <c r="G13" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H13" s="1">
         <v>4</v>
@@ -4578,7 +4578,7 @@
         <v>30</v>
       </c>
       <c r="G14" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H14" s="1">
         <v>5</v>
@@ -4604,7 +4604,7 @@
         <v>26</v>
       </c>
       <c r="G15" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15" s="1">
         <v>5</v>
@@ -4633,7 +4633,7 @@
         <v>24</v>
       </c>
       <c r="G16" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H16" s="1">
         <v>4</v>
@@ -4659,7 +4659,7 @@
         <v>24</v>
       </c>
       <c r="G17" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H17" s="1">
         <v>4</v>
@@ -4685,7 +4685,7 @@
         <v>30</v>
       </c>
       <c r="G18" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H18" s="1">
         <v>5</v>
@@ -4711,7 +4711,7 @@
         <v>26</v>
       </c>
       <c r="G19" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H19" s="1">
         <v>5</v>
@@ -4737,7 +4737,7 @@
         <v>26</v>
       </c>
       <c r="G20" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H20" s="1">
         <v>5</v>
@@ -4763,7 +4763,7 @@
         <v>30</v>
       </c>
       <c r="G21" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H21" s="1">
         <v>5</v>
@@ -4789,7 +4789,7 @@
         <v>30</v>
       </c>
       <c r="G22" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22" s="1">
         <v>5</v>
@@ -4815,7 +4815,7 @@
         <v>30</v>
       </c>
       <c r="G23" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H23" s="1">
         <v>5</v>
@@ -4841,7 +4841,7 @@
         <v>30</v>
       </c>
       <c r="G24" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H24" s="1">
         <v>5</v>
@@ -4870,7 +4870,7 @@
         <v>24</v>
       </c>
       <c r="G25" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H25" s="1">
         <v>4</v>
@@ -4896,7 +4896,7 @@
         <v>20</v>
       </c>
       <c r="G26" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H26" s="1">
         <v>4</v>
@@ -4925,7 +4925,7 @@
         <v>24</v>
       </c>
       <c r="G27" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H27" s="1">
         <v>4</v>
@@ -4951,7 +4951,7 @@
         <v>26</v>
       </c>
       <c r="G28" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H28" s="1">
         <v>5</v>
@@ -4977,7 +4977,7 @@
         <v>24</v>
       </c>
       <c r="G29" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H29" s="1">
         <v>4</v>
@@ -5003,7 +5003,7 @@
         <v>24</v>
       </c>
       <c r="G30" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H30" s="1">
         <v>4</v>
@@ -5029,7 +5029,7 @@
         <v>22</v>
       </c>
       <c r="G31" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H31" s="1">
         <v>4</v>
@@ -5055,7 +5055,7 @@
         <v>26</v>
       </c>
       <c r="G32" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H32" s="1">
         <v>5</v>
@@ -5084,7 +5084,7 @@
         <v>26</v>
       </c>
       <c r="G33" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H33" s="1">
         <v>5</v>
@@ -5113,7 +5113,7 @@
         <v>22</v>
       </c>
       <c r="G34" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H34" s="1">
         <v>4</v>
@@ -5139,7 +5139,7 @@
         <v>26</v>
       </c>
       <c r="G35" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H35" s="1">
         <v>5</v>
@@ -5165,7 +5165,7 @@
         <v>30</v>
       </c>
       <c r="G36" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H36" s="1">
         <v>5</v>
@@ -5194,7 +5194,7 @@
         <v>24</v>
       </c>
       <c r="G37" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H37" s="1">
         <v>4</v>
@@ -5220,7 +5220,7 @@
         <v>24</v>
       </c>
       <c r="G38" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H38" s="1">
         <v>4</v>
@@ -5246,7 +5246,7 @@
         <v>30</v>
       </c>
       <c r="G39" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H39" s="1">
         <v>5</v>
@@ -5275,7 +5275,7 @@
         <v>26</v>
       </c>
       <c r="G40" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H40" s="1">
         <v>5</v>
@@ -5301,7 +5301,7 @@
         <v>26</v>
       </c>
       <c r="G41" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H41" s="1">
         <v>5</v>
@@ -5327,7 +5327,7 @@
         <v>30</v>
       </c>
       <c r="G42" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H42" s="1">
         <v>5</v>
@@ -5353,7 +5353,7 @@
         <v>26</v>
       </c>
       <c r="G43" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H43" s="1">
         <v>5</v>
@@ -5379,7 +5379,7 @@
         <v>30</v>
       </c>
       <c r="G44" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H44" s="1">
         <v>5</v>
@@ -5405,7 +5405,7 @@
         <v>26</v>
       </c>
       <c r="G45" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H45" s="1">
         <v>5</v>
@@ -5431,7 +5431,7 @@
         <v>30</v>
       </c>
       <c r="G46" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="1">
         <v>5</v>
@@ -5457,7 +5457,7 @@
         <v>26</v>
       </c>
       <c r="G47" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H47" s="1">
         <v>5</v>
@@ -5483,7 +5483,7 @@
         <v>26</v>
       </c>
       <c r="G48" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H48" s="1">
         <v>5</v>
@@ -5509,7 +5509,7 @@
         <v>26</v>
       </c>
       <c r="G49" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H49" s="1">
         <v>5</v>
@@ -5535,7 +5535,7 @@
         <v>24</v>
       </c>
       <c r="G50" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H50" s="1">
         <v>4</v>
@@ -5564,7 +5564,7 @@
         <v>30</v>
       </c>
       <c r="G51" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H51" s="1">
         <v>5</v>
@@ -5590,7 +5590,7 @@
         <v>30</v>
       </c>
       <c r="G52" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H52" s="1">
         <v>5</v>
@@ -5619,7 +5619,7 @@
         <v>30</v>
       </c>
       <c r="G53" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H53" s="1">
         <v>5</v>
@@ -5648,7 +5648,7 @@
         <v>30</v>
       </c>
       <c r="G54" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H54" s="1">
         <v>5</v>
@@ -5674,7 +5674,7 @@
         <v>24</v>
       </c>
       <c r="G55" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H55" s="1">
         <v>4</v>
@@ -5700,7 +5700,7 @@
         <v>30</v>
       </c>
       <c r="G56" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H56" s="1">
         <v>5</v>
@@ -5726,7 +5726,7 @@
         <v>26</v>
       </c>
       <c r="G57" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H57" s="1">
         <v>5</v>
@@ -5752,7 +5752,7 @@
         <v>26</v>
       </c>
       <c r="G58" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H58" s="1">
         <v>5</v>
@@ -5778,7 +5778,7 @@
         <v>24</v>
       </c>
       <c r="G59" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H59" s="1">
         <v>4</v>
@@ -5804,7 +5804,7 @@
         <v>26</v>
       </c>
       <c r="G60" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H60" s="1">
         <v>5</v>
@@ -5830,7 +5830,7 @@
         <v>26</v>
       </c>
       <c r="G61" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H61" s="1">
         <v>5</v>
@@ -5856,7 +5856,7 @@
         <v>24</v>
       </c>
       <c r="G62" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H62" s="1">
         <v>4</v>
@@ -5882,7 +5882,7 @@
         <v>26</v>
       </c>
       <c r="G63" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H63" s="1">
         <v>5</v>
@@ -5908,7 +5908,7 @@
         <v>26</v>
       </c>
       <c r="G64" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H64" s="1">
         <v>5</v>
@@ -5934,7 +5934,7 @@
         <v>26</v>
       </c>
       <c r="G65" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H65" s="1">
         <v>5</v>
@@ -5960,7 +5960,7 @@
         <v>26</v>
       </c>
       <c r="G66" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H66" s="1">
         <v>5</v>
@@ -5986,7 +5986,7 @@
         <v>30</v>
       </c>
       <c r="G67" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H67" s="1">
         <v>5</v>
@@ -6015,7 +6015,7 @@
         <v>30</v>
       </c>
       <c r="G68" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H68" s="1">
         <v>5</v>
@@ -6041,7 +6041,7 @@
         <v>22</v>
       </c>
       <c r="G69" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H69" s="1">
         <v>4</v>
@@ -6067,7 +6067,7 @@
         <v>26</v>
       </c>
       <c r="G70" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H70" s="1">
         <v>5</v>
@@ -6093,7 +6093,7 @@
         <v>30</v>
       </c>
       <c r="G71" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H71" s="1">
         <v>5</v>
@@ -6119,7 +6119,7 @@
         <v>24</v>
       </c>
       <c r="G72" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H72" s="1">
         <v>4</v>
@@ -6145,7 +6145,7 @@
         <v>26</v>
       </c>
       <c r="G73" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H73" s="1">
         <v>5</v>
@@ -6171,7 +6171,7 @@
         <v>24</v>
       </c>
       <c r="G74" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H74" s="1">
         <v>4</v>
@@ -6197,7 +6197,7 @@
         <v>26</v>
       </c>
       <c r="G75" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H75" s="1">
         <v>5</v>
@@ -6223,7 +6223,7 @@
         <v>26</v>
       </c>
       <c r="G76" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H76" s="1">
         <v>5</v>
@@ -6249,7 +6249,7 @@
         <v>24</v>
       </c>
       <c r="G77" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H77" s="1">
         <v>4</v>
@@ -6275,7 +6275,7 @@
         <v>26</v>
       </c>
       <c r="G78" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H78" s="1">
         <v>5</v>
@@ -6301,7 +6301,7 @@
         <v>24</v>
       </c>
       <c r="G79" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H79" s="1">
         <v>4</v>
@@ -6327,7 +6327,7 @@
         <v>26</v>
       </c>
       <c r="G80" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H80" s="1">
         <v>5</v>
@@ -6353,7 +6353,7 @@
         <v>26</v>
       </c>
       <c r="G81" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H81" s="1">
         <v>5</v>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="G82" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H82" s="1">
         <v>4</v>
@@ -6408,7 +6408,7 @@
         <v>30</v>
       </c>
       <c r="G83" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H83" s="1">
         <v>5</v>
@@ -6434,7 +6434,7 @@
         <v>30</v>
       </c>
       <c r="G84" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H84" s="1">
         <v>5</v>
@@ -6460,7 +6460,7 @@
         <v>26</v>
       </c>
       <c r="G85" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H85" s="1">
         <v>5</v>
@@ -6489,7 +6489,7 @@
         <v>30</v>
       </c>
       <c r="G86" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H86" s="1">
         <v>5</v>
@@ -6515,7 +6515,7 @@
         <v>30</v>
       </c>
       <c r="G87" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H87" s="1">
         <v>5</v>
@@ -6541,7 +6541,7 @@
         <v>26</v>
       </c>
       <c r="G88" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H88" s="1">
         <v>5</v>
@@ -6567,7 +6567,7 @@
         <v>30</v>
       </c>
       <c r="G89" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H89" s="1">
         <v>5</v>
@@ -6596,7 +6596,7 @@
         <v>26</v>
       </c>
       <c r="G90" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H90" s="1">
         <v>5</v>
@@ -6622,7 +6622,7 @@
         <v>26</v>
       </c>
       <c r="G91" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H91" s="1">
         <v>5</v>
@@ -6648,7 +6648,7 @@
         <v>30</v>
       </c>
       <c r="G92" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H92" s="1">
         <v>5</v>
@@ -6674,7 +6674,7 @@
         <v>19</v>
       </c>
       <c r="G93" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H93" s="1">
         <v>4</v>
@@ -6700,7 +6700,7 @@
         <v>30</v>
       </c>
       <c r="G94" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H94" s="1">
         <v>5</v>
@@ -6726,7 +6726,7 @@
         <v>26</v>
       </c>
       <c r="G95" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H95" s="1">
         <v>5</v>
@@ -6752,7 +6752,7 @@
         <v>30</v>
       </c>
       <c r="G96" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H96" s="1">
         <v>5</v>
@@ -6778,7 +6778,7 @@
         <v>30</v>
       </c>
       <c r="G97" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H97" s="1">
         <v>5</v>
@@ -6804,7 +6804,7 @@
         <v>30</v>
       </c>
       <c r="G98" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H98" s="1">
         <v>5</v>
@@ -6833,7 +6833,7 @@
         <v>30</v>
       </c>
       <c r="G99" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H99" s="1">
         <v>5</v>
@@ -6859,7 +6859,7 @@
         <v>26</v>
       </c>
       <c r="G100" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H100" s="1">
         <v>5</v>
@@ -6885,7 +6885,7 @@
         <v>26</v>
       </c>
       <c r="G101" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H101" s="1">
         <v>5</v>
@@ -6911,7 +6911,7 @@
         <v>30</v>
       </c>
       <c r="G102" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H102" s="1">
         <v>5</v>
@@ -6937,7 +6937,7 @@
         <v>30</v>
       </c>
       <c r="G103" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H103" s="1">
         <v>5</v>
@@ -6966,7 +6966,7 @@
         <v>30</v>
       </c>
       <c r="G104" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H104" s="1">
         <v>5</v>
@@ -6992,7 +6992,7 @@
         <v>30</v>
       </c>
       <c r="G105" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H105" s="1">
         <v>5</v>
@@ -7018,7 +7018,7 @@
         <v>30</v>
       </c>
       <c r="G106" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H106" s="1">
         <v>5</v>
@@ -7044,7 +7044,7 @@
         <v>26</v>
       </c>
       <c r="G107" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H107" s="1">
         <v>5</v>
@@ -7070,7 +7070,7 @@
         <v>30</v>
       </c>
       <c r="G108" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H108" s="1">
         <v>5</v>
@@ -7096,7 +7096,7 @@
         <v>30</v>
       </c>
       <c r="G109" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H109" s="1">
         <v>5</v>
@@ -7122,7 +7122,7 @@
         <v>26</v>
       </c>
       <c r="G110" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H110" s="1">
         <v>5</v>
@@ -7148,7 +7148,7 @@
         <v>26</v>
       </c>
       <c r="G111" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H111" s="1">
         <v>5</v>
@@ -7174,7 +7174,7 @@
         <v>26</v>
       </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H112" s="1">
         <v>5</v>
@@ -7200,7 +7200,7 @@
         <v>26</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H113" s="1">
         <v>5</v>
@@ -7226,7 +7226,7 @@
         <v>30</v>
       </c>
       <c r="G114" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H114" s="1">
         <v>5</v>
@@ -7252,7 +7252,7 @@
         <v>30</v>
       </c>
       <c r="G115" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H115" s="1">
         <v>5</v>
@@ -7278,7 +7278,7 @@
         <v>23</v>
       </c>
       <c r="G116" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H116" s="1">
         <v>4</v>
@@ -7304,7 +7304,7 @@
         <v>24</v>
       </c>
       <c r="G117" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H117" s="1">
         <v>4</v>
@@ -7330,7 +7330,7 @@
         <v>20</v>
       </c>
       <c r="G118" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H118" s="1">
         <v>4</v>
@@ -7356,7 +7356,7 @@
         <v>26</v>
       </c>
       <c r="G119" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H119" s="1">
         <v>5</v>
@@ -7382,7 +7382,7 @@
         <v>26</v>
       </c>
       <c r="G120" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H120" s="1">
         <v>5</v>
@@ -7411,7 +7411,7 @@
         <v>30</v>
       </c>
       <c r="G121" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H121" s="1">
         <v>5</v>
@@ -7437,7 +7437,7 @@
         <v>21</v>
       </c>
       <c r="G122" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H122" s="1">
         <v>4</v>
@@ -7463,7 +7463,7 @@
         <v>30</v>
       </c>
       <c r="G123" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H123" s="1">
         <v>5</v>
@@ -7489,7 +7489,7 @@
         <v>30</v>
       </c>
       <c r="G124" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H124" s="1">
         <v>5</v>
@@ -7515,7 +7515,7 @@
         <v>30</v>
       </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H125" s="1">
         <v>5</v>
@@ -7541,7 +7541,7 @@
         <v>24</v>
       </c>
       <c r="G126" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H126" s="1">
         <v>4</v>
@@ -7567,7 +7567,7 @@
         <v>21</v>
       </c>
       <c r="G127" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H127" s="1">
         <v>4</v>
@@ -7593,7 +7593,7 @@
         <v>26</v>
       </c>
       <c r="G128" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H128" s="1">
         <v>5</v>
@@ -7619,7 +7619,7 @@
         <v>30</v>
       </c>
       <c r="G129" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H129" s="1">
         <v>5</v>
@@ -7645,7 +7645,7 @@
         <v>24</v>
       </c>
       <c r="G130" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H130" s="1">
         <v>4</v>
@@ -7671,7 +7671,7 @@
         <v>26</v>
       </c>
       <c r="G131" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H131" s="1">
         <v>5</v>
@@ -7697,7 +7697,7 @@
         <v>26</v>
       </c>
       <c r="G132" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H132" s="1">
         <v>5</v>
@@ -7726,7 +7726,7 @@
         <v>30</v>
       </c>
       <c r="G133" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H133" s="1">
         <v>5</v>
@@ -7752,7 +7752,7 @@
         <v>30</v>
       </c>
       <c r="G134" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H134" s="1">
         <v>5</v>
@@ -7778,7 +7778,7 @@
         <v>30</v>
       </c>
       <c r="G135" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H135" s="1">
         <v>5</v>
@@ -7804,7 +7804,7 @@
         <v>26</v>
       </c>
       <c r="G136" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H136" s="1">
         <v>5</v>
@@ -7830,7 +7830,7 @@
         <v>26</v>
       </c>
       <c r="G137" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H137" s="1">
         <v>5</v>
@@ -7859,7 +7859,7 @@
         <v>30</v>
       </c>
       <c r="G138" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H138" s="1">
         <v>5</v>
@@ -7885,7 +7885,7 @@
         <v>30</v>
       </c>
       <c r="G139" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H139" s="1">
         <v>5</v>
@@ -7911,7 +7911,7 @@
         <v>26</v>
       </c>
       <c r="G140" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H140" s="1">
         <v>5</v>
@@ -7937,7 +7937,7 @@
         <v>22</v>
       </c>
       <c r="G141" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H141" s="1">
         <v>4</v>
@@ -7963,7 +7963,7 @@
         <v>30</v>
       </c>
       <c r="G142" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H142" s="1">
         <v>5</v>
@@ -7989,7 +7989,7 @@
         <v>26</v>
       </c>
       <c r="G143" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H143" s="1">
         <v>5</v>
@@ -8015,7 +8015,7 @@
         <v>30</v>
       </c>
       <c r="G144" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H144" s="1">
         <v>5</v>
@@ -8041,7 +8041,7 @@
         <v>26</v>
       </c>
       <c r="G145" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H145" s="1">
         <v>5</v>
@@ -8070,7 +8070,7 @@
         <v>24</v>
       </c>
       <c r="G146" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H146" s="1">
         <v>4</v>
@@ -8099,7 +8099,7 @@
         <v>24</v>
       </c>
       <c r="G147" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H147" s="1">
         <v>4</v>
@@ -8125,7 +8125,7 @@
         <v>30</v>
       </c>
       <c r="G148" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H148" s="1">
         <v>5</v>
@@ -8151,7 +8151,7 @@
         <v>18</v>
       </c>
       <c r="G149" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H149" s="1">
         <v>3</v>
@@ -8177,7 +8177,7 @@
         <v>26</v>
       </c>
       <c r="G150" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H150" s="1">
         <v>5</v>
@@ -8206,7 +8206,7 @@
         <v>30</v>
       </c>
       <c r="G151" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H151" s="1">
         <v>5</v>
@@ -8232,7 +8232,7 @@
         <v>26</v>
       </c>
       <c r="G152" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H152" s="1">
         <v>5</v>
@@ -8258,7 +8258,7 @@
         <v>26</v>
       </c>
       <c r="G153" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H153" s="1">
         <v>5</v>
@@ -8284,7 +8284,7 @@
         <v>23</v>
       </c>
       <c r="G154" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H154" s="1">
         <v>4</v>
@@ -8310,7 +8310,7 @@
         <v>24</v>
       </c>
       <c r="G155" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H155" s="1">
         <v>4</v>
@@ -8339,7 +8339,7 @@
         <v>24</v>
       </c>
       <c r="G156" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H156" s="1">
         <v>4</v>
@@ -8365,7 +8365,7 @@
         <v>30</v>
       </c>
       <c r="G157" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H157" s="1">
         <v>5</v>
@@ -10280,6 +10280,153 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
+    <col min="3" max="5" width="19.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>431</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>432</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>434</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>435</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>436</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <ignoredErrors>
+    <ignoredError sqref="C4:C6 C2:C3 C7:C8" twoDigitTextYear="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C1037"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -21703,7 +21850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D90FE78-749D-4E79-8923-ED8BD0B01BA1}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -21771,7 +21918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -22886,153 +23033,6 @@
   </sheetData>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="25.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
-    <col min="3" max="5" width="19.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B2" s="1">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>431</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>432</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>433</v>
-      </c>
-      <c r="B5" s="1">
-        <v>2</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>434</v>
-      </c>
-      <c r="B6" s="1">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>435</v>
-      </c>
-      <c r="B7" s="1">
-        <v>2</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>436</v>
-      </c>
-      <c r="B8" s="1">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <ignoredErrors>
-    <ignoredError sqref="C4:C6 C2:C3 C7:C8" twoDigitTextYear="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: correção da inserção de planejamento individual e regra d máximo de dias para o professor.
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CCF78F-7D5C-4212-8E99-BF6A923D9655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF73A01B-2E92-42CE-A956-5FF2477D8F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1633,7 +1633,8 @@
         <v>114</v>
       </c>
       <c r="B2" s="1">
-        <v>300</v>
+        <f>30*60</f>
+        <v>1800</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: Correção do dashboard para impressã correta do resultado e porcentagem de agrupamento dos componentes.
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF73A01B-2E92-42CE-A956-5FF2477D8F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF47324-B04E-48EF-B56A-4528FB7BAE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1633,8 +1633,8 @@
         <v>114</v>
       </c>
       <c r="B2" s="1">
-        <f>30*60</f>
-        <v>1800</v>
+        <f>10*60</f>
+        <v>600</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>